<commit_message>
Add Superior logo to checklist header
</commit_message>
<xml_diff>
--- a/New_Hire_Orientation_Checklist.xlsx
+++ b/New_Hire_Orientation_Checklist.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,7 +28,12 @@
     <font>
       <b val="1"/>
       <color rgb="001e293b"/>
-      <sz val="14"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00f59e0b"/>
+      <sz val="11"/>
     </font>
     <font>
       <i val="1"/>
@@ -90,14 +95,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -109,7 +124,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -184,6 +199,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1809750" cy="495300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -475,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -485,282 +530,297 @@
     <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>SUPERIOR HUNTINGDON COMPOSITES — NEW HIRE ORIENTATION CHECKLIST</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Complete all items in order. New hire may NOT work ANY task solo until Phase 2 sign-offs are complete.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="1" ht="27" customHeight="1"/>
+    <row r="2" ht="27" customHeight="1"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>NEW HIRE ORIENTATION CHECKLIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Superior Huntingdon Composites, LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="10" customHeight="1"/>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>⚠ Complete all items IN ORDER. No solo work on ANY task until Phase 2 sign-offs complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Phase / Item</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Trainer Initials</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>PHASE 1 — DAY 1: SAFETY FOUNDATIONS</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Site tour — emergency exits, muster points, alarms, eyewash/shower, extinguishers, first aid</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-    </row>
-    <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="C10" s="9" t="n"/>
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="8" t="n"/>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>PPE requirements per area</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-    </row>
-    <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="8" t="n"/>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>HazCom / SDS binder location</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr"/>
-      <c r="D8" s="7" t="inlineStr"/>
-      <c r="E8" s="6" t="inlineStr"/>
-    </row>
-    <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="8" t="n"/>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>How to report a hazard or near miss — and that it is safe to report</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr"/>
-      <c r="D9" s="7" t="inlineStr"/>
-      <c r="E9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="C13" s="9" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="8" t="n"/>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Assigned trainer / mentor confirmed</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr"/>
-      <c r="D10" s="7" t="inlineStr"/>
-      <c r="E10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="C14" s="9" t="n"/>
+      <c r="D14" s="9" t="n"/>
+      <c r="E14" s="8" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>PHASE 2 — WEEKS 1-2: SHADOW + TASK SIGN-OFF</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>JSA walkthrough of each core task with trainer</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr"/>
-      <c r="D12" s="7" t="inlineStr"/>
-      <c r="E12" s="6" t="inlineStr"/>
-    </row>
-    <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="C16" s="9" t="n"/>
+      <c r="D16" s="9" t="n"/>
+      <c r="E16" s="8" t="n"/>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Trainee demonstrates each core task under direct observation</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr"/>
-      <c r="D13" s="7" t="inlineStr"/>
-      <c r="E13" s="6" t="inlineStr"/>
-    </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="C17" s="9" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="8" t="n"/>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Trainer signs off EACH task individually (not one blanket sign-off)</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr"/>
-      <c r="D14" s="7" t="inlineStr"/>
-      <c r="E14" s="6" t="inlineStr"/>
-    </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="C18" s="9" t="n"/>
+      <c r="D18" s="9" t="n"/>
+      <c r="E18" s="8" t="n"/>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>GATE: No solo work on any task until signed off</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr"/>
-      <c r="D15" s="7" t="inlineStr"/>
-      <c r="E15" s="6" t="inlineStr"/>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="C19" s="9" t="n"/>
+      <c r="D19" s="9" t="n"/>
+      <c r="E19" s="8" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>PHASE 3 — WEEKS 3-4: VERIFY</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>30-day competency check with trainer</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr"/>
-      <c r="D17" s="7" t="inlineStr"/>
-      <c r="E17" s="6" t="inlineStr"/>
-    </row>
-    <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="C21" s="9" t="n"/>
+      <c r="D21" s="9" t="n"/>
+      <c r="E21" s="8" t="n"/>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Debrief — any hazards noticed during first weeks?</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr"/>
-      <c r="D18" s="7" t="inlineStr"/>
-      <c r="E18" s="6" t="inlineStr"/>
-    </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="C22" s="9" t="n"/>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="8" t="n"/>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>Confirm new hire is working independently and safely</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr"/>
-      <c r="D19" s="7" t="inlineStr"/>
-      <c r="E19" s="6" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="8" t="inlineStr">
+      <c r="C23" s="9" t="n"/>
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="8" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>New Hire Name:</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="8" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>Hire Date:</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="8" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>Trainer Signature:</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="8" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>Supervisor / EHS Review:</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A5:E5"/>
+  <mergeCells count="7">
+    <mergeCell ref="A1:D2"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>